<commit_message>
fix the auth guard and set up the route protection
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9885" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9885"/>
   </bookViews>
   <sheets>
     <sheet name="tasks" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="347">
   <si>
     <t>Module</t>
   </si>
@@ -1169,6 +1169,9 @@
   </si>
   <si>
     <t>Westerns</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
   </si>
 </sst>
 </file>
@@ -1651,7 +1654,10 @@
         <v>75</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>74</v>
+        <v>346</v>
+      </c>
+      <c r="E2" s="1">
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1709,7 +1715,7 @@
         <v>75</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>74</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
passes user data to the header component
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="346">
   <si>
     <t>Module</t>
   </si>
@@ -46,9 +46,6 @@
   </si>
   <si>
     <t xml:space="preserve">checks if the email exist before resetting the password </t>
-  </si>
-  <si>
-    <t>Remove header and footer in the login/signup pages and only show them for login user</t>
   </si>
   <si>
     <t>Displays certain field of the header only for authenticated users</t>
@@ -1171,7 +1168,7 @@
     <t>Westerns</t>
   </si>
   <si>
-    <t>Ongoing</t>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -1615,7 +1612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.5703125" style="3" customWidth="1"/>
@@ -1634,13 +1631,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1651,13 +1648,13 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E2" s="1">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1666,10 +1663,10 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>74</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1678,22 +1675,21 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>74</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1701,62 +1697,53 @@
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D8" s="1" t="s">
-        <v>74</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>9</v>
-      </c>
+      <c r="A11" s="19"/>
       <c r="B11" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="19"/>
       <c r="B12" s="1" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1765,10 +1752,10 @@
         <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1777,10 +1764,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1788,39 +1775,38 @@
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
-      <c r="B16" s="1" t="s">
-        <v>13</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="C17" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
@@ -1828,26 +1814,26 @@
         <v>14</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
+      <c r="D20" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="C21" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D21" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.3">
@@ -1855,10 +1841,10 @@
         <v>16</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
@@ -1866,10 +1852,10 @@
         <v>17</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
@@ -1877,10 +1863,10 @@
         <v>18</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
@@ -1888,10 +1874,10 @@
         <v>19</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
@@ -1899,10 +1885,10 @@
         <v>20</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
@@ -1910,26 +1896,26 @@
         <v>21</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="1" t="s">
+      <c r="D28" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="C29" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D29" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
@@ -1937,10 +1923,10 @@
         <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
@@ -1948,10 +1934,10 @@
         <v>24</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
@@ -1959,10 +1945,10 @@
         <v>25</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
@@ -1970,10 +1956,10 @@
         <v>26</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
@@ -1981,76 +1967,76 @@
         <v>27</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B37" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B37" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
-      <c r="B38" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C38" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B40" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
@@ -2058,10 +2044,10 @@
         <v>34</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
@@ -2069,10 +2055,10 @@
         <v>35</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
@@ -2080,37 +2066,37 @@
         <v>36</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B44" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B44" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="45" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
-      <c r="B45" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D45" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B46" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="C46" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D46" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
@@ -2118,10 +2104,10 @@
         <v>39</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
@@ -2129,10 +2115,10 @@
         <v>40</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -2140,10 +2126,10 @@
         <v>41</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
@@ -2151,21 +2137,21 @@
         <v>42</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B51" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B52" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>74</v>
+      <c r="C52" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
@@ -2173,10 +2159,10 @@
         <v>44</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
@@ -2184,10 +2170,10 @@
         <v>45</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -2195,35 +2181,36 @@
         <v>46</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A58" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C56" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>74</v>
+      <c r="B58" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="19"/>
+      <c r="B59" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B59" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="C59" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2232,10 +2219,10 @@
         <v>49</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2244,10 +2231,10 @@
         <v>50</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2256,10 +2243,10 @@
         <v>51</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2268,55 +2255,54 @@
         <v>52</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="19"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B66" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B67" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
@@ -2324,10 +2310,10 @@
         <v>57</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
@@ -2335,29 +2321,29 @@
         <v>58</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="1" t="s">
+      <c r="C70" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B71" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C70" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C71" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -2365,35 +2351,36 @@
         <v>60</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B73" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A74" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C73" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>74</v>
+      <c r="B74" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75" s="19" t="s">
+      <c r="A75" s="19"/>
+      <c r="B75" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="C75" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2402,22 +2389,22 @@
         <v>63</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="19"/>
       <c r="B77" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2426,10 +2413,10 @@
         <v>66</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2438,47 +2425,35 @@
         <v>67</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="19"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B81" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A75:A80"/>
-    <mergeCell ref="A59:A64"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A11:A16"/>
+    <mergeCell ref="A74:A79"/>
+    <mergeCell ref="A58:A63"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A10:A15"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C81">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C80">
       <formula1>"Low,Medium,Urgent,Immediate"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D81">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D80">
       <formula1>"Not started, Ongoing,Tested,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2512,19 +2487,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
         <v>80</v>
       </c>
-      <c r="C1" t="s">
-        <v>81</v>
-      </c>
       <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
         <v>72</v>
       </c>
-      <c r="E1" t="s">
-        <v>73</v>
-      </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2544,41 +2519,41 @@
   <sheetData>
     <row r="1" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="9"/>
       <c r="D2" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="9"/>
       <c r="D3" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="9"/>
@@ -2586,7 +2561,7 @@
     </row>
     <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="9"/>
@@ -2594,7 +2569,7 @@
     </row>
     <row r="6" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="9"/>
@@ -2602,7 +2577,7 @@
     </row>
     <row r="7" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="9"/>
@@ -2610,7 +2585,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9"/>
@@ -2618,7 +2593,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
@@ -2626,7 +2601,7 @@
     </row>
     <row r="10" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9"/>
@@ -2634,7 +2609,7 @@
     </row>
     <row r="11" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
@@ -2642,7 +2617,7 @@
     </row>
     <row r="12" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
@@ -2650,7 +2625,7 @@
     </row>
     <row r="13" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
@@ -2658,7 +2633,7 @@
     </row>
     <row r="14" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
@@ -2666,7 +2641,7 @@
     </row>
     <row r="15" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
@@ -2674,7 +2649,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
@@ -2682,7 +2657,7 @@
     </row>
     <row r="17" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
@@ -2690,7 +2665,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
@@ -2698,7 +2673,7 @@
     </row>
     <row r="19" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
@@ -2706,7 +2681,7 @@
     </row>
     <row r="20" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
@@ -2714,7 +2689,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
@@ -2722,7 +2697,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
@@ -2730,7 +2705,7 @@
     </row>
     <row r="23" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
@@ -2738,7 +2713,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
@@ -2746,7 +2721,7 @@
     </row>
     <row r="25" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
@@ -2754,7 +2729,7 @@
     </row>
     <row r="26" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="9"/>
@@ -2762,7 +2737,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
@@ -2770,7 +2745,7 @@
     </row>
     <row r="28" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
@@ -2778,7 +2753,7 @@
     </row>
     <row r="29" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
@@ -2786,7 +2761,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="9"/>
@@ -2794,7 +2769,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
@@ -2802,7 +2777,7 @@
     </row>
     <row r="32" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
@@ -2810,7 +2785,7 @@
     </row>
     <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
@@ -2818,7 +2793,7 @@
     </row>
     <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="9"/>
@@ -2826,7 +2801,7 @@
     </row>
     <row r="35" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
@@ -2834,7 +2809,7 @@
     </row>
     <row r="36" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="9"/>
@@ -2842,7 +2817,7 @@
     </row>
     <row r="37" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="9"/>
@@ -2850,7 +2825,7 @@
     </row>
     <row r="38" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
@@ -2858,7 +2833,7 @@
     </row>
     <row r="39" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B39" s="8"/>
       <c r="C39" s="9"/>
@@ -2866,7 +2841,7 @@
     </row>
     <row r="40" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="9"/>
@@ -2874,7 +2849,7 @@
     </row>
     <row r="41" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B41" s="8"/>
       <c r="C41" s="9"/>
@@ -2882,7 +2857,7 @@
     </row>
     <row r="42" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="9"/>
@@ -2890,7 +2865,7 @@
     </row>
     <row r="43" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B43" s="8"/>
       <c r="C43" s="9"/>
@@ -2898,7 +2873,7 @@
     </row>
     <row r="44" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="9"/>
@@ -2906,7 +2881,7 @@
     </row>
     <row r="45" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="9"/>
@@ -2914,7 +2889,7 @@
     </row>
     <row r="46" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B46" s="8"/>
       <c r="C46" s="9"/>
@@ -2922,7 +2897,7 @@
     </row>
     <row r="47" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="9"/>
@@ -2930,7 +2905,7 @@
     </row>
     <row r="48" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B48" s="8"/>
       <c r="C48" s="9"/>
@@ -2938,7 +2913,7 @@
     </row>
     <row r="49" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="9"/>
@@ -2946,7 +2921,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B50" s="8"/>
       <c r="C50" s="9"/>
@@ -2954,7 +2929,7 @@
     </row>
     <row r="51" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="9"/>
@@ -2962,7 +2937,7 @@
     </row>
     <row r="52" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B52" s="8"/>
       <c r="C52" s="9"/>
@@ -2970,7 +2945,7 @@
     </row>
     <row r="53" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B53" s="8"/>
       <c r="C53" s="9"/>
@@ -2978,7 +2953,7 @@
     </row>
     <row r="54" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="9"/>
@@ -2986,7 +2961,7 @@
     </row>
     <row r="55" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B55" s="8"/>
       <c r="C55" s="9"/>
@@ -2994,7 +2969,7 @@
     </row>
     <row r="56" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="9"/>
@@ -3002,7 +2977,7 @@
     </row>
     <row r="57" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
@@ -3010,7 +2985,7 @@
     </row>
     <row r="58" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="9"/>
@@ -3018,7 +2993,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B59" s="8"/>
       <c r="C59" s="9"/>
@@ -3026,7 +3001,7 @@
     </row>
     <row r="60" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="9"/>
@@ -3034,7 +3009,7 @@
     </row>
     <row r="61" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B61" s="8"/>
       <c r="C61" s="9"/>
@@ -3042,7 +3017,7 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="9"/>
@@ -3050,7 +3025,7 @@
     </row>
     <row r="63" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>
@@ -3058,7 +3033,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="9"/>
@@ -3066,7 +3041,7 @@
     </row>
     <row r="65" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B65" s="8"/>
       <c r="C65" s="9"/>
@@ -3074,7 +3049,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="9"/>
@@ -3082,7 +3057,7 @@
     </row>
     <row r="67" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B67" s="8"/>
       <c r="C67" s="9"/>
@@ -3090,7 +3065,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B68" s="8"/>
       <c r="C68" s="9"/>
@@ -3098,7 +3073,7 @@
     </row>
     <row r="69" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B69" s="8"/>
       <c r="C69" s="9"/>
@@ -3106,7 +3081,7 @@
     </row>
     <row r="70" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B70" s="8"/>
       <c r="C70" s="9"/>
@@ -3114,7 +3089,7 @@
     </row>
     <row r="71" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B71" s="8"/>
       <c r="C71" s="9"/>
@@ -3122,7 +3097,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B72" s="8"/>
       <c r="C72" s="9"/>
@@ -3130,7 +3105,7 @@
     </row>
     <row r="73" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B73" s="8"/>
       <c r="C73" s="9"/>
@@ -3138,7 +3113,7 @@
     </row>
     <row r="74" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B74" s="8"/>
       <c r="C74" s="9"/>
@@ -3146,7 +3121,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B75" s="8"/>
       <c r="C75" s="9"/>
@@ -3154,7 +3129,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B76" s="8"/>
       <c r="C76" s="9"/>
@@ -3162,7 +3137,7 @@
     </row>
     <row r="77" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B77" s="8"/>
       <c r="C77" s="9"/>
@@ -3170,7 +3145,7 @@
     </row>
     <row r="78" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B78" s="8"/>
       <c r="C78" s="9"/>
@@ -3178,7 +3153,7 @@
     </row>
     <row r="79" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B79" s="8"/>
       <c r="C79" s="9"/>
@@ -3186,7 +3161,7 @@
     </row>
     <row r="80" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B80" s="8"/>
       <c r="C80" s="9"/>
@@ -3194,7 +3169,7 @@
     </row>
     <row r="81" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B81" s="8"/>
       <c r="C81" s="9"/>
@@ -3202,7 +3177,7 @@
     </row>
     <row r="82" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B82" s="8"/>
       <c r="C82" s="9"/>
@@ -3210,7 +3185,7 @@
     </row>
     <row r="83" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B83" s="8"/>
       <c r="C83" s="9"/>
@@ -3218,7 +3193,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B84" s="8"/>
       <c r="C84" s="9"/>
@@ -3226,7 +3201,7 @@
     </row>
     <row r="85" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B85" s="8"/>
       <c r="C85" s="9"/>
@@ -3234,7 +3209,7 @@
     </row>
     <row r="86" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B86" s="8"/>
       <c r="C86" s="9"/>
@@ -3242,7 +3217,7 @@
     </row>
     <row r="87" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B87" s="8"/>
       <c r="C87" s="9"/>
@@ -3250,7 +3225,7 @@
     </row>
     <row r="88" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B88" s="8"/>
       <c r="C88" s="9"/>
@@ -3258,7 +3233,7 @@
     </row>
     <row r="89" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B89" s="8"/>
       <c r="C89" s="9"/>
@@ -3266,7 +3241,7 @@
     </row>
     <row r="90" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B90" s="8"/>
       <c r="C90" s="9"/>
@@ -3274,7 +3249,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B91" s="8"/>
       <c r="C91" s="9"/>
@@ -3282,7 +3257,7 @@
     </row>
     <row r="92" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B92" s="8"/>
       <c r="C92" s="9"/>
@@ -3290,7 +3265,7 @@
     </row>
     <row r="93" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B93" s="8"/>
       <c r="C93" s="9"/>
@@ -3298,7 +3273,7 @@
     </row>
     <row r="94" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B94" s="8"/>
       <c r="C94" s="9"/>
@@ -3306,7 +3281,7 @@
     </row>
     <row r="95" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="9"/>
@@ -3314,7 +3289,7 @@
     </row>
     <row r="96" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B96" s="8"/>
       <c r="C96" s="9"/>
@@ -3322,7 +3297,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="9"/>
@@ -3330,7 +3305,7 @@
     </row>
     <row r="98" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B98" s="8"/>
       <c r="C98" s="9"/>
@@ -3338,7 +3313,7 @@
     </row>
     <row r="99" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B99" s="8"/>
       <c r="C99" s="9"/>
@@ -3346,7 +3321,7 @@
     </row>
     <row r="100" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B100" s="8"/>
       <c r="C100" s="9"/>
@@ -3354,7 +3329,7 @@
     </row>
     <row r="101" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B101" s="8"/>
       <c r="C101" s="9"/>
@@ -3362,7 +3337,7 @@
     </row>
     <row r="102" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B102" s="8"/>
       <c r="C102" s="9"/>
@@ -3370,7 +3345,7 @@
     </row>
     <row r="103" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B103" s="8"/>
       <c r="C103" s="9"/>
@@ -3378,7 +3353,7 @@
     </row>
     <row r="104" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B104" s="8"/>
       <c r="C104" s="9"/>
@@ -3386,7 +3361,7 @@
     </row>
     <row r="105" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B105" s="8"/>
       <c r="C105" s="9"/>
@@ -3394,7 +3369,7 @@
     </row>
     <row r="106" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B106" s="8"/>
       <c r="C106" s="9"/>
@@ -3402,7 +3377,7 @@
     </row>
     <row r="107" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B107" s="8"/>
       <c r="C107" s="9"/>
@@ -3410,7 +3385,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B108" s="8"/>
       <c r="C108" s="9"/>
@@ -3418,7 +3393,7 @@
     </row>
     <row r="109" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B109" s="8"/>
       <c r="C109" s="9"/>
@@ -3426,7 +3401,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B110" s="8"/>
       <c r="C110" s="9"/>
@@ -3434,7 +3409,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B111" s="8"/>
       <c r="C111" s="9"/>
@@ -3442,7 +3417,7 @@
     </row>
     <row r="112" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B112" s="8"/>
       <c r="C112" s="9"/>
@@ -3450,7 +3425,7 @@
     </row>
     <row r="113" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="9"/>
@@ -3458,7 +3433,7 @@
     </row>
     <row r="114" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B114" s="8"/>
       <c r="C114" s="9"/>
@@ -3466,7 +3441,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B115" s="8"/>
       <c r="C115" s="9"/>
@@ -3474,7 +3449,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B116" s="8"/>
       <c r="C116" s="9"/>
@@ -3482,7 +3457,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B117" s="8"/>
       <c r="C117" s="9"/>
@@ -3490,7 +3465,7 @@
     </row>
     <row r="118" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B118" s="8"/>
       <c r="C118" s="9"/>
@@ -3498,7 +3473,7 @@
     </row>
     <row r="119" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B119" s="8"/>
       <c r="C119" s="9"/>
@@ -3506,7 +3481,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B120" s="8"/>
       <c r="C120" s="9"/>
@@ -3514,7 +3489,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B121" s="8"/>
       <c r="C121" s="9"/>
@@ -3522,7 +3497,7 @@
     </row>
     <row r="122" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B122" s="8"/>
       <c r="C122" s="9"/>
@@ -3530,7 +3505,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B123" s="8"/>
       <c r="C123" s="9"/>
@@ -3538,7 +3513,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B124" s="8"/>
       <c r="C124" s="9"/>
@@ -3546,7 +3521,7 @@
     </row>
     <row r="125" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B125" s="8"/>
       <c r="C125" s="9"/>
@@ -3554,7 +3529,7 @@
     </row>
     <row r="126" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B126" s="8"/>
       <c r="C126" s="9"/>
@@ -3562,7 +3537,7 @@
     </row>
     <row r="127" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B127" s="8"/>
       <c r="C127" s="9"/>
@@ -3570,7 +3545,7 @@
     </row>
     <row r="128" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B128" s="8"/>
       <c r="C128" s="9"/>
@@ -3578,7 +3553,7 @@
     </row>
     <row r="129" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B129" s="8"/>
       <c r="C129" s="9"/>
@@ -3586,7 +3561,7 @@
     </row>
     <row r="130" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B130" s="8"/>
       <c r="C130" s="9"/>
@@ -3594,7 +3569,7 @@
     </row>
     <row r="131" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B131" s="8"/>
       <c r="C131" s="9"/>
@@ -3602,7 +3577,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B132" s="8"/>
       <c r="C132" s="9"/>
@@ -3610,7 +3585,7 @@
     </row>
     <row r="133" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B133" s="8"/>
       <c r="C133" s="9"/>
@@ -3618,7 +3593,7 @@
     </row>
     <row r="134" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B134" s="8"/>
       <c r="C134" s="9"/>
@@ -3626,7 +3601,7 @@
     </row>
     <row r="135" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B135" s="8"/>
       <c r="C135" s="9"/>
@@ -3634,7 +3609,7 @@
     </row>
     <row r="136" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B136" s="8"/>
       <c r="C136" s="9"/>
@@ -3642,7 +3617,7 @@
     </row>
     <row r="137" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B137" s="8"/>
       <c r="C137" s="9"/>
@@ -3650,7 +3625,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B138" s="8"/>
       <c r="C138" s="9"/>
@@ -3658,7 +3633,7 @@
     </row>
     <row r="139" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B139" s="8"/>
       <c r="C139" s="9"/>
@@ -3666,7 +3641,7 @@
     </row>
     <row r="140" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B140" s="8"/>
       <c r="C140" s="9"/>
@@ -3674,7 +3649,7 @@
     </row>
     <row r="141" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B141" s="8"/>
       <c r="C141" s="9"/>
@@ -3682,7 +3657,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B142" s="8"/>
       <c r="C142" s="9"/>
@@ -3690,7 +3665,7 @@
     </row>
     <row r="143" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B143" s="8"/>
       <c r="C143" s="9"/>
@@ -3698,7 +3673,7 @@
     </row>
     <row r="144" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B144" s="8"/>
       <c r="C144" s="9"/>
@@ -3706,7 +3681,7 @@
     </row>
     <row r="145" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B145" s="8"/>
       <c r="C145" s="9"/>
@@ -3714,7 +3689,7 @@
     </row>
     <row r="146" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B146" s="8"/>
       <c r="C146" s="9"/>
@@ -3722,7 +3697,7 @@
     </row>
     <row r="147" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B147" s="8"/>
       <c r="C147" s="9"/>
@@ -3730,7 +3705,7 @@
     </row>
     <row r="148" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A148" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B148" s="8"/>
       <c r="C148" s="9"/>
@@ -3738,7 +3713,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B149" s="8"/>
       <c r="C149" s="9"/>
@@ -3746,7 +3721,7 @@
     </row>
     <row r="150" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B150" s="8"/>
       <c r="C150" s="9"/>
@@ -3754,7 +3729,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B151" s="8"/>
       <c r="C151" s="9"/>
@@ -3762,7 +3737,7 @@
     </row>
     <row r="152" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B152" s="8"/>
       <c r="C152" s="9"/>
@@ -3770,7 +3745,7 @@
     </row>
     <row r="153" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A153" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B153" s="8"/>
       <c r="C153" s="9"/>
@@ -3778,7 +3753,7 @@
     </row>
     <row r="154" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B154" s="8"/>
       <c r="C154" s="9"/>
@@ -3786,7 +3761,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B155" s="8"/>
       <c r="C155" s="9"/>
@@ -3794,7 +3769,7 @@
     </row>
     <row r="156" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B156" s="8"/>
       <c r="C156" s="9"/>
@@ -3802,7 +3777,7 @@
     </row>
     <row r="157" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B157" s="8"/>
       <c r="C157" s="9"/>
@@ -3810,7 +3785,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B158" s="8"/>
       <c r="C158" s="9"/>
@@ -3818,7 +3793,7 @@
     </row>
     <row r="159" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B159" s="8"/>
       <c r="C159" s="9"/>
@@ -3826,7 +3801,7 @@
     </row>
     <row r="160" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B160" s="8"/>
       <c r="C160" s="9"/>
@@ -3834,7 +3809,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B161" s="8"/>
       <c r="C161" s="9"/>
@@ -3842,7 +3817,7 @@
     </row>
     <row r="162" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B162" s="8"/>
       <c r="C162" s="9"/>
@@ -3850,7 +3825,7 @@
     </row>
     <row r="163" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B163" s="8"/>
       <c r="C163" s="9"/>
@@ -3858,7 +3833,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B164" s="8"/>
       <c r="C164" s="9"/>
@@ -3866,7 +3841,7 @@
     </row>
     <row r="165" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A165" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B165" s="8"/>
       <c r="C165" s="9"/>
@@ -3874,7 +3849,7 @@
     </row>
     <row r="166" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B166" s="8"/>
       <c r="C166" s="9"/>
@@ -3882,7 +3857,7 @@
     </row>
     <row r="167" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B167" s="8"/>
       <c r="C167" s="9"/>
@@ -3890,7 +3865,7 @@
     </row>
     <row r="168" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B168" s="8"/>
       <c r="C168" s="9"/>
@@ -3898,7 +3873,7 @@
     </row>
     <row r="169" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B169" s="8"/>
       <c r="C169" s="9"/>
@@ -3906,7 +3881,7 @@
     </row>
     <row r="170" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B170" s="8"/>
       <c r="C170" s="9"/>
@@ -3914,7 +3889,7 @@
     </row>
     <row r="171" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A171" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B171" s="8"/>
       <c r="C171" s="9"/>
@@ -3922,7 +3897,7 @@
     </row>
     <row r="172" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B172" s="8"/>
       <c r="C172" s="9"/>
@@ -3930,7 +3905,7 @@
     </row>
     <row r="173" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B173" s="8"/>
       <c r="C173" s="9"/>
@@ -3938,7 +3913,7 @@
     </row>
     <row r="174" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B174" s="8"/>
       <c r="C174" s="9"/>
@@ -3946,7 +3921,7 @@
     </row>
     <row r="175" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B175" s="8"/>
       <c r="C175" s="9"/>
@@ -3954,7 +3929,7 @@
     </row>
     <row r="176" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A176" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B176" s="8"/>
       <c r="C176" s="9"/>
@@ -3962,7 +3937,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B177" s="8"/>
       <c r="C177" s="9"/>
@@ -3970,7 +3945,7 @@
     </row>
     <row r="178" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B178" s="8"/>
       <c r="C178" s="9"/>
@@ -3978,7 +3953,7 @@
     </row>
     <row r="179" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A179" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B179" s="8"/>
       <c r="C179" s="9"/>
@@ -3986,7 +3961,7 @@
     </row>
     <row r="180" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B180" s="8"/>
       <c r="C180" s="9"/>
@@ -3994,7 +3969,7 @@
     </row>
     <row r="181" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A181" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B181" s="8"/>
       <c r="C181" s="9"/>
@@ -4002,7 +3977,7 @@
     </row>
     <row r="182" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A182" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B182" s="8"/>
       <c r="C182" s="9"/>
@@ -4010,7 +3985,7 @@
     </row>
     <row r="183" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B183" s="8"/>
       <c r="C183" s="9"/>
@@ -4018,7 +3993,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B184" s="8"/>
       <c r="C184" s="9"/>
@@ -4026,7 +4001,7 @@
     </row>
     <row r="185" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B185" s="8"/>
       <c r="C185" s="9"/>
@@ -4034,7 +4009,7 @@
     </row>
     <row r="186" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A186" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B186" s="8"/>
       <c r="C186" s="9"/>
@@ -4042,7 +4017,7 @@
     </row>
     <row r="187" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B187" s="8"/>
       <c r="C187" s="9"/>
@@ -4050,7 +4025,7 @@
     </row>
     <row r="188" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B188" s="8"/>
       <c r="C188" s="9"/>
@@ -4058,7 +4033,7 @@
     </row>
     <row r="189" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A189" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B189" s="8"/>
       <c r="C189" s="9"/>
@@ -4066,7 +4041,7 @@
     </row>
     <row r="190" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A190" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B190" s="8"/>
       <c r="C190" s="9"/>
@@ -4074,7 +4049,7 @@
     </row>
     <row r="191" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A191" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B191" s="8"/>
       <c r="C191" s="9"/>
@@ -4082,7 +4057,7 @@
     </row>
     <row r="192" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A192" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B192" s="8"/>
       <c r="C192" s="9"/>
@@ -4090,7 +4065,7 @@
     </row>
     <row r="193" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A193" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B193" s="8"/>
       <c r="C193" s="9"/>
@@ -4098,7 +4073,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B194" s="8"/>
       <c r="C194" s="9"/>
@@ -4106,7 +4081,7 @@
     </row>
     <row r="195" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B195" s="8"/>
       <c r="C195" s="9"/>
@@ -4114,7 +4089,7 @@
     </row>
     <row r="196" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B196" s="8"/>
       <c r="C196" s="9"/>
@@ -4122,7 +4097,7 @@
     </row>
     <row r="197" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B197" s="8"/>
       <c r="C197" s="9"/>
@@ -4130,7 +4105,7 @@
     </row>
     <row r="198" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B198" s="8"/>
       <c r="C198" s="9"/>
@@ -4138,7 +4113,7 @@
     </row>
     <row r="199" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B199" s="8"/>
       <c r="C199" s="9"/>
@@ -4146,7 +4121,7 @@
     </row>
     <row r="200" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B200" s="8"/>
       <c r="C200" s="9"/>
@@ -4154,7 +4129,7 @@
     </row>
     <row r="201" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B201" s="8"/>
       <c r="C201" s="9"/>
@@ -4162,7 +4137,7 @@
     </row>
     <row r="202" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B202" s="8"/>
       <c r="C202" s="9"/>
@@ -4170,7 +4145,7 @@
     </row>
     <row r="203" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B203" s="8"/>
       <c r="C203" s="9"/>
@@ -4178,7 +4153,7 @@
     </row>
     <row r="204" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B204" s="8"/>
       <c r="C204" s="9"/>
@@ -4186,7 +4161,7 @@
     </row>
     <row r="205" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B205" s="8"/>
       <c r="C205" s="9"/>
@@ -4194,7 +4169,7 @@
     </row>
     <row r="206" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B206" s="8"/>
       <c r="C206" s="9"/>
@@ -4202,7 +4177,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B207" s="8"/>
       <c r="C207" s="9"/>
@@ -4228,146 +4203,146 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" t="s">
         <v>84</v>
       </c>
-      <c r="B1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>85</v>
       </c>
-      <c r="E1" t="s">
-        <v>86</v>
-      </c>
       <c r="F1" s="16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>313</v>
-      </c>
       <c r="F4" s="16" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F5" s="16" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F6" s="17"/>
     </row>
     <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="C8" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F10" s="16" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F11" s="16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F12" s="16" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F13" s="16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F14" s="16" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F16" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F17" s="16" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F18" s="16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F19" s="16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -4375,44 +4350,44 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F21" s="18" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -4420,47 +4395,47 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F28" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F29" s="18" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F31" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F32" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="33" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F33" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="34" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F34" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="36" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F36" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="37" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F37" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
filled the dropdown with data from json
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="347">
   <si>
     <t>Module</t>
   </si>
@@ -1169,6 +1169,9 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>Auth module completed</t>
   </si>
 </sst>
 </file>
@@ -1703,6 +1706,11 @@
         <v>345</v>
       </c>
     </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E7" s="1" t="s">
+        <v>346</v>
+      </c>
+    </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
added fe logic for agent management
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="348">
   <si>
     <t>Module</t>
   </si>
@@ -1174,7 +1174,7 @@
     <t>Auth module completed</t>
   </si>
   <si>
-    <t>Ongoing</t>
+    <t>contact.vlcam.net@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1760,7 +1760,7 @@
         <v>75</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1784,7 +1784,7 @@
         <v>75</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -1799,10 +1799,10 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="19"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>70</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>15</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>16</v>
       </c>
@@ -1856,8 +1856,11 @@
       <c r="D22" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="16" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1868,7 +1871,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>18</v>
       </c>
@@ -1879,7 +1882,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>19</v>
       </c>
@@ -1890,7 +1893,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>20</v>
       </c>
@@ -1901,7 +1904,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
         <v>21</v>
       </c>
@@ -1912,7 +1915,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
@@ -1923,7 +1926,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
         <v>23</v>
       </c>
@@ -1934,7 +1937,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
         <v>24</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
         <v>25</v>
       </c>
@@ -2460,8 +2463,11 @@
       <formula1>"Not started, Ongoing,Tested,Done"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E22" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update the models and the form for rdv insertion
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="349">
   <si>
     <t>Module</t>
   </si>
@@ -1175,6 +1175,9 @@
   </si>
   <si>
     <t>contact.vlcam.net@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">they do not connect no need to delete them </t>
   </si>
 </sst>
 </file>
@@ -1798,6 +1801,9 @@
       <c r="D15" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="E15" s="1" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="19"/>
@@ -1810,7 +1816,7 @@
         <v>75</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
@@ -1821,7 +1827,7 @@
         <v>75</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
@@ -1832,7 +1838,7 @@
         <v>75</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
@@ -1843,7 +1849,7 @@
         <v>75</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
@@ -1854,7 +1860,7 @@
         <v>75</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
       <c r="E22" s="16" t="s">
         <v>347</v>
@@ -1868,7 +1874,7 @@
         <v>75</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
@@ -1879,7 +1885,7 @@
         <v>75</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
@@ -1890,7 +1896,7 @@
         <v>75</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
@@ -1901,7 +1907,7 @@
         <v>75</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
add,delete comment view article
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="355">
   <si>
     <t>Module</t>
   </si>
@@ -229,9 +229,6 @@
   </si>
   <si>
     <t xml:space="preserve">Make the website bilingual and give the user the possibility to choose </t>
-  </si>
-  <si>
-    <t>Fix the image upload and make it possible for the user to upload profile picture and image</t>
   </si>
   <si>
     <t>add valid links in the footer for social media button</t>
@@ -1178,6 +1175,27 @@
   </si>
   <si>
     <t xml:space="preserve">they do not connect no need to delete them </t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>sanitize socials url  before saving</t>
+  </si>
+  <si>
+    <t>rejected</t>
+  </si>
+  <si>
+    <t>Fix the image upload and make it possible for the user to upload blog picture and image</t>
+  </si>
+  <si>
+    <t>send email to user when he subscribe to a rdv</t>
+  </si>
+  <si>
+    <t>gener</t>
+  </si>
+  <si>
+    <t>send review email to user, generate  a review with link</t>
   </si>
 </sst>
 </file>
@@ -1624,7 +1642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.5703125" style="3" customWidth="1"/>
@@ -1632,10 +1650,11 @@
     <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="23.140625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="28.85546875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1643,16 +1662,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>2</v>
       </c>
@@ -1660,163 +1679,169 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E2" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="F2" s="1" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="20"/>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="20"/>
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E7" s="1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E7" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="20"/>
       <c r="B11" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="20"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="20"/>
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="20"/>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="20"/>
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="19"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
@@ -1824,10 +1849,10 @@
         <v>13</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
@@ -1835,10 +1860,10 @@
         <v>14</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
@@ -1846,10 +1871,10 @@
         <v>15</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
@@ -1857,13 +1882,13 @@
         <v>16</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
@@ -1871,10 +1896,10 @@
         <v>17</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
@@ -1882,10 +1907,10 @@
         <v>18</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
@@ -1893,10 +1918,10 @@
         <v>19</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
@@ -1904,10 +1929,10 @@
         <v>20</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
@@ -1915,10 +1940,10 @@
         <v>21</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
@@ -1926,10 +1951,10 @@
         <v>22</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
@@ -1937,10 +1962,10 @@
         <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
@@ -1948,10 +1973,10 @@
         <v>24</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
@@ -1959,10 +1984,10 @@
         <v>25</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
@@ -1970,10 +1995,10 @@
         <v>26</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
@@ -1981,10 +2006,10 @@
         <v>27</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
@@ -1992,10 +2017,10 @@
         <v>29</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
@@ -2003,10 +2028,10 @@
         <v>28</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
@@ -2014,10 +2039,10 @@
         <v>32</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
@@ -2025,10 +2050,10 @@
         <v>30</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
@@ -2036,10 +2061,10 @@
         <v>31</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
@@ -2047,10 +2072,10 @@
         <v>33</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
@@ -2058,10 +2083,10 @@
         <v>34</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
@@ -2069,10 +2094,10 @@
         <v>35</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
@@ -2080,10 +2105,10 @@
         <v>36</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
@@ -2091,10 +2116,10 @@
         <v>37</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
@@ -2105,10 +2130,10 @@
         <v>38</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
@@ -2116,10 +2141,10 @@
         <v>39</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
@@ -2127,79 +2152,82 @@
         <v>40</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B49" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B50" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B52" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B53" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B54" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B55" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="20" t="s">
         <v>47</v>
       </c>
@@ -2207,81 +2235,81 @@
         <v>64</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="20"/>
       <c r="B59" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="20"/>
       <c r="B60" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="20"/>
       <c r="B61" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="20"/>
       <c r="B62" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="20"/>
       <c r="B63" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>73</v>
+        <v>344</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
@@ -2289,10 +2317,10 @@
         <v>55</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
@@ -2300,10 +2328,10 @@
         <v>54</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
@@ -2311,10 +2339,10 @@
         <v>56</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
@@ -2322,10 +2350,10 @@
         <v>57</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
@@ -2333,18 +2361,18 @@
         <v>58</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C70" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
@@ -2352,10 +2380,10 @@
         <v>59</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -2363,10 +2391,10 @@
         <v>60</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2374,13 +2402,13 @@
         <v>61</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2389,10 +2417,10 @@
         <v>62</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2401,10 +2429,10 @@
         <v>63</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2413,10 +2441,10 @@
         <v>65</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2425,33 +2453,48 @@
         <v>66</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="20"/>
       <c r="B79" s="1" t="s">
-        <v>67</v>
+        <v>351</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B81" s="1" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B82" s="1" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B83" s="1" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -2502,19 +2545,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" t="s">
         <v>79</v>
       </c>
-      <c r="C1" t="s">
-        <v>80</v>
-      </c>
       <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
         <v>71</v>
       </c>
-      <c r="E1" t="s">
-        <v>72</v>
-      </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2534,41 +2577,41 @@
   <sheetData>
     <row r="1" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>81</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="9"/>
       <c r="D2" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="9"/>
       <c r="D3" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="9"/>
@@ -2576,7 +2619,7 @@
     </row>
     <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="9"/>
@@ -2584,7 +2627,7 @@
     </row>
     <row r="6" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="9"/>
@@ -2592,7 +2635,7 @@
     </row>
     <row r="7" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="9"/>
@@ -2600,7 +2643,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9"/>
@@ -2608,7 +2651,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="9"/>
@@ -2616,7 +2659,7 @@
     </row>
     <row r="10" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9"/>
@@ -2624,7 +2667,7 @@
     </row>
     <row r="11" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
@@ -2632,7 +2675,7 @@
     </row>
     <row r="12" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
@@ -2640,7 +2683,7 @@
     </row>
     <row r="13" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
@@ -2648,7 +2691,7 @@
     </row>
     <row r="14" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
@@ -2656,7 +2699,7 @@
     </row>
     <row r="15" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
@@ -2664,7 +2707,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
@@ -2672,7 +2715,7 @@
     </row>
     <row r="17" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
@@ -2680,7 +2723,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
@@ -2688,7 +2731,7 @@
     </row>
     <row r="19" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
@@ -2696,7 +2739,7 @@
     </row>
     <row r="20" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
@@ -2704,7 +2747,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
@@ -2712,7 +2755,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
@@ -2720,7 +2763,7 @@
     </row>
     <row r="23" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
@@ -2728,7 +2771,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
@@ -2736,7 +2779,7 @@
     </row>
     <row r="25" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
@@ -2744,7 +2787,7 @@
     </row>
     <row r="26" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="9"/>
@@ -2752,7 +2795,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
@@ -2760,7 +2803,7 @@
     </row>
     <row r="28" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
@@ -2768,7 +2811,7 @@
     </row>
     <row r="29" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
@@ -2776,7 +2819,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="9"/>
@@ -2784,7 +2827,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
@@ -2792,7 +2835,7 @@
     </row>
     <row r="32" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
@@ -2800,7 +2843,7 @@
     </row>
     <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
@@ -2808,7 +2851,7 @@
     </row>
     <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="9"/>
@@ -2816,7 +2859,7 @@
     </row>
     <row r="35" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
@@ -2824,7 +2867,7 @@
     </row>
     <row r="36" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="9"/>
@@ -2832,7 +2875,7 @@
     </row>
     <row r="37" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="9"/>
@@ -2840,7 +2883,7 @@
     </row>
     <row r="38" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
@@ -2848,7 +2891,7 @@
     </row>
     <row r="39" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B39" s="8"/>
       <c r="C39" s="9"/>
@@ -2856,7 +2899,7 @@
     </row>
     <row r="40" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="9"/>
@@ -2864,7 +2907,7 @@
     </row>
     <row r="41" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B41" s="8"/>
       <c r="C41" s="9"/>
@@ -2872,7 +2915,7 @@
     </row>
     <row r="42" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="9"/>
@@ -2880,7 +2923,7 @@
     </row>
     <row r="43" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B43" s="8"/>
       <c r="C43" s="9"/>
@@ -2888,7 +2931,7 @@
     </row>
     <row r="44" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="9"/>
@@ -2896,7 +2939,7 @@
     </row>
     <row r="45" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="9"/>
@@ -2904,7 +2947,7 @@
     </row>
     <row r="46" spans="1:4" ht="71.25" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B46" s="8"/>
       <c r="C46" s="9"/>
@@ -2912,7 +2955,7 @@
     </row>
     <row r="47" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="9"/>
@@ -2920,7 +2963,7 @@
     </row>
     <row r="48" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B48" s="8"/>
       <c r="C48" s="9"/>
@@ -2928,7 +2971,7 @@
     </row>
     <row r="49" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="9"/>
@@ -2936,7 +2979,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B50" s="8"/>
       <c r="C50" s="9"/>
@@ -2944,7 +2987,7 @@
     </row>
     <row r="51" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="9"/>
@@ -2952,7 +2995,7 @@
     </row>
     <row r="52" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B52" s="8"/>
       <c r="C52" s="9"/>
@@ -2960,7 +3003,7 @@
     </row>
     <row r="53" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B53" s="8"/>
       <c r="C53" s="9"/>
@@ -2968,7 +3011,7 @@
     </row>
     <row r="54" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="9"/>
@@ -2976,7 +3019,7 @@
     </row>
     <row r="55" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B55" s="8"/>
       <c r="C55" s="9"/>
@@ -2984,7 +3027,7 @@
     </row>
     <row r="56" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="9"/>
@@ -2992,7 +3035,7 @@
     </row>
     <row r="57" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
@@ -3000,7 +3043,7 @@
     </row>
     <row r="58" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="9"/>
@@ -3008,7 +3051,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B59" s="8"/>
       <c r="C59" s="9"/>
@@ -3016,7 +3059,7 @@
     </row>
     <row r="60" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="9"/>
@@ -3024,7 +3067,7 @@
     </row>
     <row r="61" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B61" s="8"/>
       <c r="C61" s="9"/>
@@ -3032,7 +3075,7 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="9"/>
@@ -3040,7 +3083,7 @@
     </row>
     <row r="63" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>
@@ -3048,7 +3091,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="9"/>
@@ -3056,7 +3099,7 @@
     </row>
     <row r="65" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B65" s="8"/>
       <c r="C65" s="9"/>
@@ -3064,7 +3107,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="9"/>
@@ -3072,7 +3115,7 @@
     </row>
     <row r="67" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B67" s="8"/>
       <c r="C67" s="9"/>
@@ -3080,7 +3123,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B68" s="8"/>
       <c r="C68" s="9"/>
@@ -3088,7 +3131,7 @@
     </row>
     <row r="69" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B69" s="8"/>
       <c r="C69" s="9"/>
@@ -3096,7 +3139,7 @@
     </row>
     <row r="70" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B70" s="8"/>
       <c r="C70" s="9"/>
@@ -3104,7 +3147,7 @@
     </row>
     <row r="71" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B71" s="8"/>
       <c r="C71" s="9"/>
@@ -3112,7 +3155,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B72" s="8"/>
       <c r="C72" s="9"/>
@@ -3120,7 +3163,7 @@
     </row>
     <row r="73" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B73" s="8"/>
       <c r="C73" s="9"/>
@@ -3128,7 +3171,7 @@
     </row>
     <row r="74" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B74" s="8"/>
       <c r="C74" s="9"/>
@@ -3136,7 +3179,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B75" s="8"/>
       <c r="C75" s="9"/>
@@ -3144,7 +3187,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B76" s="8"/>
       <c r="C76" s="9"/>
@@ -3152,7 +3195,7 @@
     </row>
     <row r="77" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B77" s="8"/>
       <c r="C77" s="9"/>
@@ -3160,7 +3203,7 @@
     </row>
     <row r="78" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B78" s="8"/>
       <c r="C78" s="9"/>
@@ -3168,7 +3211,7 @@
     </row>
     <row r="79" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B79" s="8"/>
       <c r="C79" s="9"/>
@@ -3176,7 +3219,7 @@
     </row>
     <row r="80" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B80" s="8"/>
       <c r="C80" s="9"/>
@@ -3184,7 +3227,7 @@
     </row>
     <row r="81" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B81" s="8"/>
       <c r="C81" s="9"/>
@@ -3192,7 +3235,7 @@
     </row>
     <row r="82" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B82" s="8"/>
       <c r="C82" s="9"/>
@@ -3200,7 +3243,7 @@
     </row>
     <row r="83" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B83" s="8"/>
       <c r="C83" s="9"/>
@@ -3208,7 +3251,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B84" s="8"/>
       <c r="C84" s="9"/>
@@ -3216,7 +3259,7 @@
     </row>
     <row r="85" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B85" s="8"/>
       <c r="C85" s="9"/>
@@ -3224,7 +3267,7 @@
     </row>
     <row r="86" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B86" s="8"/>
       <c r="C86" s="9"/>
@@ -3232,7 +3275,7 @@
     </row>
     <row r="87" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B87" s="8"/>
       <c r="C87" s="9"/>
@@ -3240,7 +3283,7 @@
     </row>
     <row r="88" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B88" s="8"/>
       <c r="C88" s="9"/>
@@ -3248,7 +3291,7 @@
     </row>
     <row r="89" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B89" s="8"/>
       <c r="C89" s="9"/>
@@ -3256,7 +3299,7 @@
     </row>
     <row r="90" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B90" s="8"/>
       <c r="C90" s="9"/>
@@ -3264,7 +3307,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B91" s="8"/>
       <c r="C91" s="9"/>
@@ -3272,7 +3315,7 @@
     </row>
     <row r="92" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B92" s="8"/>
       <c r="C92" s="9"/>
@@ -3280,7 +3323,7 @@
     </row>
     <row r="93" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B93" s="8"/>
       <c r="C93" s="9"/>
@@ -3288,7 +3331,7 @@
     </row>
     <row r="94" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B94" s="8"/>
       <c r="C94" s="9"/>
@@ -3296,7 +3339,7 @@
     </row>
     <row r="95" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="9"/>
@@ -3304,7 +3347,7 @@
     </row>
     <row r="96" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B96" s="8"/>
       <c r="C96" s="9"/>
@@ -3312,7 +3355,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="9"/>
@@ -3320,7 +3363,7 @@
     </row>
     <row r="98" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B98" s="8"/>
       <c r="C98" s="9"/>
@@ -3328,7 +3371,7 @@
     </row>
     <row r="99" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B99" s="8"/>
       <c r="C99" s="9"/>
@@ -3336,7 +3379,7 @@
     </row>
     <row r="100" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B100" s="8"/>
       <c r="C100" s="9"/>
@@ -3344,7 +3387,7 @@
     </row>
     <row r="101" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B101" s="8"/>
       <c r="C101" s="9"/>
@@ -3352,7 +3395,7 @@
     </row>
     <row r="102" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B102" s="8"/>
       <c r="C102" s="9"/>
@@ -3360,7 +3403,7 @@
     </row>
     <row r="103" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B103" s="8"/>
       <c r="C103" s="9"/>
@@ -3368,7 +3411,7 @@
     </row>
     <row r="104" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B104" s="8"/>
       <c r="C104" s="9"/>
@@ -3376,7 +3419,7 @@
     </row>
     <row r="105" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B105" s="8"/>
       <c r="C105" s="9"/>
@@ -3384,7 +3427,7 @@
     </row>
     <row r="106" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B106" s="8"/>
       <c r="C106" s="9"/>
@@ -3392,7 +3435,7 @@
     </row>
     <row r="107" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B107" s="8"/>
       <c r="C107" s="9"/>
@@ -3400,7 +3443,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B108" s="8"/>
       <c r="C108" s="9"/>
@@ -3408,7 +3451,7 @@
     </row>
     <row r="109" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B109" s="8"/>
       <c r="C109" s="9"/>
@@ -3416,7 +3459,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B110" s="8"/>
       <c r="C110" s="9"/>
@@ -3424,7 +3467,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B111" s="8"/>
       <c r="C111" s="9"/>
@@ -3432,7 +3475,7 @@
     </row>
     <row r="112" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B112" s="8"/>
       <c r="C112" s="9"/>
@@ -3440,7 +3483,7 @@
     </row>
     <row r="113" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="9"/>
@@ -3448,7 +3491,7 @@
     </row>
     <row r="114" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B114" s="8"/>
       <c r="C114" s="9"/>
@@ -3456,7 +3499,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B115" s="8"/>
       <c r="C115" s="9"/>
@@ -3464,7 +3507,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B116" s="8"/>
       <c r="C116" s="9"/>
@@ -3472,7 +3515,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B117" s="8"/>
       <c r="C117" s="9"/>
@@ -3480,7 +3523,7 @@
     </row>
     <row r="118" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B118" s="8"/>
       <c r="C118" s="9"/>
@@ -3488,7 +3531,7 @@
     </row>
     <row r="119" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B119" s="8"/>
       <c r="C119" s="9"/>
@@ -3496,7 +3539,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B120" s="8"/>
       <c r="C120" s="9"/>
@@ -3504,7 +3547,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B121" s="8"/>
       <c r="C121" s="9"/>
@@ -3512,7 +3555,7 @@
     </row>
     <row r="122" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B122" s="8"/>
       <c r="C122" s="9"/>
@@ -3520,7 +3563,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B123" s="8"/>
       <c r="C123" s="9"/>
@@ -3528,7 +3571,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B124" s="8"/>
       <c r="C124" s="9"/>
@@ -3536,7 +3579,7 @@
     </row>
     <row r="125" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B125" s="8"/>
       <c r="C125" s="9"/>
@@ -3544,7 +3587,7 @@
     </row>
     <row r="126" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B126" s="8"/>
       <c r="C126" s="9"/>
@@ -3552,7 +3595,7 @@
     </row>
     <row r="127" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B127" s="8"/>
       <c r="C127" s="9"/>
@@ -3560,7 +3603,7 @@
     </row>
     <row r="128" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B128" s="8"/>
       <c r="C128" s="9"/>
@@ -3568,7 +3611,7 @@
     </row>
     <row r="129" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B129" s="8"/>
       <c r="C129" s="9"/>
@@ -3576,7 +3619,7 @@
     </row>
     <row r="130" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B130" s="8"/>
       <c r="C130" s="9"/>
@@ -3584,7 +3627,7 @@
     </row>
     <row r="131" spans="1:4" ht="57" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B131" s="8"/>
       <c r="C131" s="9"/>
@@ -3592,7 +3635,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B132" s="8"/>
       <c r="C132" s="9"/>
@@ -3600,7 +3643,7 @@
     </row>
     <row r="133" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B133" s="8"/>
       <c r="C133" s="9"/>
@@ -3608,7 +3651,7 @@
     </row>
     <row r="134" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B134" s="8"/>
       <c r="C134" s="9"/>
@@ -3616,7 +3659,7 @@
     </row>
     <row r="135" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B135" s="8"/>
       <c r="C135" s="9"/>
@@ -3624,7 +3667,7 @@
     </row>
     <row r="136" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B136" s="8"/>
       <c r="C136" s="9"/>
@@ -3632,7 +3675,7 @@
     </row>
     <row r="137" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B137" s="8"/>
       <c r="C137" s="9"/>
@@ -3640,7 +3683,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B138" s="8"/>
       <c r="C138" s="9"/>
@@ -3648,7 +3691,7 @@
     </row>
     <row r="139" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B139" s="8"/>
       <c r="C139" s="9"/>
@@ -3656,7 +3699,7 @@
     </row>
     <row r="140" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B140" s="8"/>
       <c r="C140" s="9"/>
@@ -3664,7 +3707,7 @@
     </row>
     <row r="141" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B141" s="8"/>
       <c r="C141" s="9"/>
@@ -3672,7 +3715,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B142" s="8"/>
       <c r="C142" s="9"/>
@@ -3680,7 +3723,7 @@
     </row>
     <row r="143" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B143" s="8"/>
       <c r="C143" s="9"/>
@@ -3688,7 +3731,7 @@
     </row>
     <row r="144" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B144" s="8"/>
       <c r="C144" s="9"/>
@@ -3696,7 +3739,7 @@
     </row>
     <row r="145" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B145" s="8"/>
       <c r="C145" s="9"/>
@@ -3704,7 +3747,7 @@
     </row>
     <row r="146" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B146" s="8"/>
       <c r="C146" s="9"/>
@@ -3712,7 +3755,7 @@
     </row>
     <row r="147" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B147" s="8"/>
       <c r="C147" s="9"/>
@@ -3720,7 +3763,7 @@
     </row>
     <row r="148" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A148" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B148" s="8"/>
       <c r="C148" s="9"/>
@@ -3728,7 +3771,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B149" s="8"/>
       <c r="C149" s="9"/>
@@ -3736,7 +3779,7 @@
     </row>
     <row r="150" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B150" s="8"/>
       <c r="C150" s="9"/>
@@ -3744,7 +3787,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B151" s="8"/>
       <c r="C151" s="9"/>
@@ -3752,7 +3795,7 @@
     </row>
     <row r="152" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B152" s="8"/>
       <c r="C152" s="9"/>
@@ -3760,7 +3803,7 @@
     </row>
     <row r="153" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A153" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B153" s="8"/>
       <c r="C153" s="9"/>
@@ -3768,7 +3811,7 @@
     </row>
     <row r="154" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B154" s="8"/>
       <c r="C154" s="9"/>
@@ -3776,7 +3819,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B155" s="8"/>
       <c r="C155" s="9"/>
@@ -3784,7 +3827,7 @@
     </row>
     <row r="156" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B156" s="8"/>
       <c r="C156" s="9"/>
@@ -3792,7 +3835,7 @@
     </row>
     <row r="157" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B157" s="8"/>
       <c r="C157" s="9"/>
@@ -3800,7 +3843,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B158" s="8"/>
       <c r="C158" s="9"/>
@@ -3808,7 +3851,7 @@
     </row>
     <row r="159" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B159" s="8"/>
       <c r="C159" s="9"/>
@@ -3816,7 +3859,7 @@
     </row>
     <row r="160" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B160" s="8"/>
       <c r="C160" s="9"/>
@@ -3824,7 +3867,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B161" s="8"/>
       <c r="C161" s="9"/>
@@ -3832,7 +3875,7 @@
     </row>
     <row r="162" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B162" s="8"/>
       <c r="C162" s="9"/>
@@ -3840,7 +3883,7 @@
     </row>
     <row r="163" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B163" s="8"/>
       <c r="C163" s="9"/>
@@ -3848,7 +3891,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B164" s="8"/>
       <c r="C164" s="9"/>
@@ -3856,7 +3899,7 @@
     </row>
     <row r="165" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A165" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B165" s="8"/>
       <c r="C165" s="9"/>
@@ -3864,7 +3907,7 @@
     </row>
     <row r="166" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B166" s="8"/>
       <c r="C166" s="9"/>
@@ -3872,7 +3915,7 @@
     </row>
     <row r="167" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B167" s="8"/>
       <c r="C167" s="9"/>
@@ -3880,7 +3923,7 @@
     </row>
     <row r="168" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B168" s="8"/>
       <c r="C168" s="9"/>
@@ -3888,7 +3931,7 @@
     </row>
     <row r="169" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B169" s="8"/>
       <c r="C169" s="9"/>
@@ -3896,7 +3939,7 @@
     </row>
     <row r="170" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B170" s="8"/>
       <c r="C170" s="9"/>
@@ -3904,7 +3947,7 @@
     </row>
     <row r="171" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A171" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B171" s="8"/>
       <c r="C171" s="9"/>
@@ -3912,7 +3955,7 @@
     </row>
     <row r="172" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B172" s="8"/>
       <c r="C172" s="9"/>
@@ -3920,7 +3963,7 @@
     </row>
     <row r="173" spans="1:4" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B173" s="8"/>
       <c r="C173" s="9"/>
@@ -3928,7 +3971,7 @@
     </row>
     <row r="174" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B174" s="8"/>
       <c r="C174" s="9"/>
@@ -3936,7 +3979,7 @@
     </row>
     <row r="175" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B175" s="8"/>
       <c r="C175" s="9"/>
@@ -3944,7 +3987,7 @@
     </row>
     <row r="176" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A176" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B176" s="8"/>
       <c r="C176" s="9"/>
@@ -3952,7 +3995,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B177" s="8"/>
       <c r="C177" s="9"/>
@@ -3960,7 +4003,7 @@
     </row>
     <row r="178" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B178" s="8"/>
       <c r="C178" s="9"/>
@@ -3968,7 +4011,7 @@
     </row>
     <row r="179" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A179" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B179" s="8"/>
       <c r="C179" s="9"/>
@@ -3976,7 +4019,7 @@
     </row>
     <row r="180" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B180" s="8"/>
       <c r="C180" s="9"/>
@@ -3984,7 +4027,7 @@
     </row>
     <row r="181" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A181" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B181" s="8"/>
       <c r="C181" s="9"/>
@@ -3992,7 +4035,7 @@
     </row>
     <row r="182" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A182" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B182" s="8"/>
       <c r="C182" s="9"/>
@@ -4000,7 +4043,7 @@
     </row>
     <row r="183" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B183" s="8"/>
       <c r="C183" s="9"/>
@@ -4008,7 +4051,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B184" s="8"/>
       <c r="C184" s="9"/>
@@ -4016,7 +4059,7 @@
     </row>
     <row r="185" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B185" s="8"/>
       <c r="C185" s="9"/>
@@ -4024,7 +4067,7 @@
     </row>
     <row r="186" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A186" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B186" s="8"/>
       <c r="C186" s="9"/>
@@ -4032,7 +4075,7 @@
     </row>
     <row r="187" spans="1:4" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B187" s="8"/>
       <c r="C187" s="9"/>
@@ -4040,7 +4083,7 @@
     </row>
     <row r="188" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B188" s="8"/>
       <c r="C188" s="9"/>
@@ -4048,7 +4091,7 @@
     </row>
     <row r="189" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A189" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B189" s="8"/>
       <c r="C189" s="9"/>
@@ -4056,7 +4099,7 @@
     </row>
     <row r="190" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A190" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B190" s="8"/>
       <c r="C190" s="9"/>
@@ -4064,7 +4107,7 @@
     </row>
     <row r="191" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A191" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B191" s="8"/>
       <c r="C191" s="9"/>
@@ -4072,7 +4115,7 @@
     </row>
     <row r="192" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A192" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B192" s="8"/>
       <c r="C192" s="9"/>
@@ -4080,7 +4123,7 @@
     </row>
     <row r="193" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A193" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B193" s="8"/>
       <c r="C193" s="9"/>
@@ -4088,7 +4131,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B194" s="8"/>
       <c r="C194" s="9"/>
@@ -4096,7 +4139,7 @@
     </row>
     <row r="195" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B195" s="8"/>
       <c r="C195" s="9"/>
@@ -4104,7 +4147,7 @@
     </row>
     <row r="196" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B196" s="8"/>
       <c r="C196" s="9"/>
@@ -4112,7 +4155,7 @@
     </row>
     <row r="197" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B197" s="8"/>
       <c r="C197" s="9"/>
@@ -4120,7 +4163,7 @@
     </row>
     <row r="198" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B198" s="8"/>
       <c r="C198" s="9"/>
@@ -4128,7 +4171,7 @@
     </row>
     <row r="199" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B199" s="8"/>
       <c r="C199" s="9"/>
@@ -4136,7 +4179,7 @@
     </row>
     <row r="200" spans="1:4" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B200" s="8"/>
       <c r="C200" s="9"/>
@@ -4144,7 +4187,7 @@
     </row>
     <row r="201" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B201" s="8"/>
       <c r="C201" s="9"/>
@@ -4152,7 +4195,7 @@
     </row>
     <row r="202" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B202" s="8"/>
       <c r="C202" s="9"/>
@@ -4160,7 +4203,7 @@
     </row>
     <row r="203" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B203" s="8"/>
       <c r="C203" s="9"/>
@@ -4168,7 +4211,7 @@
     </row>
     <row r="204" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B204" s="8"/>
       <c r="C204" s="9"/>
@@ -4176,7 +4219,7 @@
     </row>
     <row r="205" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B205" s="8"/>
       <c r="C205" s="9"/>
@@ -4184,7 +4227,7 @@
     </row>
     <row r="206" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B206" s="8"/>
       <c r="C206" s="9"/>
@@ -4192,7 +4235,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B207" s="8"/>
       <c r="C207" s="9"/>
@@ -4218,146 +4261,146 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" t="s">
         <v>83</v>
       </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
-        <v>85</v>
-      </c>
       <c r="F1" s="16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>312</v>
-      </c>
       <c r="F4" s="16" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F5" s="16" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F6" s="17"/>
     </row>
     <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="C8" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F10" s="16" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F11" s="16" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F12" s="16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F13" s="16" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F14" s="16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F16" s="16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F17" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F18" s="16" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F19" s="16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -4365,44 +4408,44 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F21" s="18" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -4410,47 +4453,47 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F28" s="18" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F29" s="18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F31" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F32" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="33" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F33" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="34" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F34" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="36" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F36" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="37" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F37" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
loaded the dasbord metrics data and styled the page
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="388">
   <si>
     <t>Module</t>
   </si>
@@ -1271,6 +1271,30 @@
   </si>
   <si>
     <t>montant total gagner par mois</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t>NOTIFICATIONS</t>
+  </si>
+  <si>
+    <t>create a model for notification</t>
+  </si>
+  <si>
+    <t>create a notification for prestation personalise</t>
+  </si>
+  <si>
+    <t>list all the notifications</t>
+  </si>
+  <si>
+    <t>update the notification using a cron job</t>
+  </si>
+  <si>
+    <t>resolve a notification</t>
+  </si>
+  <si>
+    <t>archive notification after a certain time to free the database</t>
   </si>
 </sst>
 </file>
@@ -1717,7 +1741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.5703125" style="3" customWidth="1"/>
@@ -2084,7 +2108,7 @@
         <v>74</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.3">
@@ -2095,7 +2119,7 @@
         <v>74</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.3">
@@ -2106,7 +2130,7 @@
         <v>74</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>72</v>
+        <v>380</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
@@ -2117,7 +2141,7 @@
         <v>74</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
@@ -2128,7 +2152,7 @@
         <v>74</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
@@ -2139,7 +2163,7 @@
         <v>74</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
@@ -2150,7 +2174,7 @@
         <v>74</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
@@ -2161,7 +2185,7 @@
         <v>74</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
@@ -2183,7 +2207,7 @@
         <v>74</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
@@ -2194,7 +2218,7 @@
         <v>74</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
@@ -2208,7 +2232,7 @@
         <v>74</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
@@ -2219,7 +2243,7 @@
         <v>74</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
@@ -2230,7 +2254,7 @@
         <v>74</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -2241,7 +2265,7 @@
         <v>74</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -2252,7 +2276,7 @@
         <v>74</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -2313,7 +2337,7 @@
         <v>74</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2325,7 +2349,7 @@
         <v>74</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2349,7 +2373,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2361,7 +2385,7 @@
         <v>74</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2495,7 +2519,7 @@
         <v>74</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2507,7 +2531,7 @@
         <v>74</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>72</v>
+        <v>344</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2554,40 +2578,76 @@
         <v>74</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B81" s="1" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C81" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B82" s="1" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C82" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B83" s="1" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C83" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B84" s="1" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C84" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B85" s="1" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C85" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B86" s="1" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C86" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>358</v>
       </c>
@@ -2595,32 +2655,32 @@
         <v>359</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B91" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B92" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B93" s="1" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
         <v>365</v>
       </c>
@@ -2693,9 +2753,42 @@
         <v>378</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
         <v>379</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B116" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B117" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B118" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B119" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B120" s="1" t="s">
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2706,10 +2799,10 @@
     <mergeCell ref="A10:A15"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C80">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C86">
       <formula1>"Low,Medium,Urgent,Immediate"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D80">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D86">
       <formula1>"Not started, Ongoing,Tested,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
added table data to the dashbord component
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="388">
   <si>
     <t>Module</t>
   </si>
@@ -2130,7 +2130,7 @@
         <v>74</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>380</v>
+        <v>344</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
@@ -2685,110 +2685,161 @@
         <v>365</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B98" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
         <v>368</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D102" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B103" s="1" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D103" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B104" s="1" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D104" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D105" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B106" s="1" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D106" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B107" s="1" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D107" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B108" s="1" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D108" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D109" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D110" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D111" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B112" s="1" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D112" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
         <v>381</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D115" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B116" s="1" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D116" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B117" s="1" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D117" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B118" s="1" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D118" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B119" s="1" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D119" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B120" s="1" t="s">
         <v>387</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2802,7 +2853,7 @@
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C86">
       <formula1>"Low,Medium,Urgent,Immediate"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D86">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D86 D102:D112 D115:D120">
       <formula1>"Not started, Ongoing,Tested,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
added models and methods for notifications,create a notification
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="388">
   <si>
     <t>Module</t>
   </si>
@@ -1231,12 +1231,6 @@
     <t>refine the blog module</t>
   </si>
   <si>
-    <t>page prise de rdv</t>
-  </si>
-  <si>
-    <t>video prise de rdv</t>
-  </si>
-  <si>
     <t>service performance</t>
   </si>
   <si>
@@ -1295,6 +1289,12 @@
   </si>
   <si>
     <t>archive notification after a certain time to free the database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implement the like functionality </t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload images </t>
   </si>
 </sst>
 </file>
@@ -2578,7 +2578,7 @@
         <v>74</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>344</v>
+        <v>378</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
@@ -2654,53 +2654,80 @@
       <c r="B90" s="1" t="s">
         <v>359</v>
       </c>
+      <c r="D90" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B91" s="1" t="s">
         <v>360</v>
       </c>
+      <c r="D91" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B92" s="1" t="s">
         <v>361</v>
       </c>
+      <c r="D92" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B93" s="1" t="s">
         <v>362</v>
       </c>
+      <c r="D93" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
         <v>363</v>
       </c>
+      <c r="D94" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
         <v>364</v>
       </c>
+      <c r="D95" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
         <v>365</v>
       </c>
+      <c r="D96" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
-        <v>366</v>
+        <v>386</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B98" s="1" t="s">
-        <v>367</v>
+        <v>387</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D102" s="1" t="s">
         <v>344</v>
@@ -2708,7 +2735,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B103" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>344</v>
@@ -2716,7 +2743,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B104" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D104" s="1" t="s">
         <v>344</v>
@@ -2724,7 +2751,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>344</v>
@@ -2732,7 +2759,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B106" s="1" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D106" s="1" t="s">
         <v>344</v>
@@ -2740,7 +2767,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B107" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D107" s="1" t="s">
         <v>344</v>
@@ -2748,7 +2775,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B108" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>344</v>
@@ -2756,7 +2783,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D109" s="1" t="s">
         <v>344</v>
@@ -2764,23 +2791,23 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>380</v>
+        <v>344</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>380</v>
+        <v>344</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B112" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D112" s="1" t="s">
         <v>344</v>
@@ -2788,15 +2815,15 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D115" s="1" t="s">
         <v>72</v>
@@ -2804,7 +2831,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B116" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>72</v>
@@ -2812,7 +2839,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B117" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>72</v>
@@ -2820,7 +2847,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B118" s="1" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D118" s="1" t="s">
         <v>72</v>
@@ -2828,7 +2855,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B119" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>72</v>
@@ -2836,7 +2863,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B120" s="1" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D120" s="1" t="s">
         <v>72</v>
@@ -2853,7 +2880,7 @@
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="Priority" sqref="C2:C86">
       <formula1>"Low,Medium,Urgent,Immediate"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D86 D102:D112 D115:D120">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D86 D102:D112 D115:D120 D90:D98">
       <formula1>"Not started, Ongoing,Tested,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
...some changes on notifications
</commit_message>
<xml_diff>
--- a/franny-finals-task.xlsx
+++ b/franny-finals-task.xlsx
@@ -2711,7 +2711,7 @@
         <v>386</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>344</v>
+        <v>378</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
@@ -2719,7 +2719,7 @@
         <v>387</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>344</v>
+        <v>72</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>